<commit_message>
Scrape 2026-09-22 - rapport off-cycle / summer
</commit_message>
<xml_diff>
--- a/data/stages_finance_marche.xlsx
+++ b/data/stages_finance_marche.xlsx
@@ -517,7 +517,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mis a jour le 22/09/2026 a 12:25 UTC</t>
+          <t>Mis a jour le 22/09/2026 a 12:35 UTC</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>4974</v>
+        <v>4978</v>
       </c>
     </row>
     <row r="42">

</xml_diff>